<commit_message>
Update Tram B Data Set
</commit_message>
<xml_diff>
--- a/Bordeaux_DigitalTwin_Documentation.xlsx
+++ b/Bordeaux_DigitalTwin_Documentation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Master M2\InterShhip\Dashboard\bordeaux_twin_final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_70C4458D53CF42AF874505EB22EE58A6D06D0A3F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{51F1794D-5AEA-40F3-8DF6-8C5D2FACACE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="817" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">AirQuality!$A$1:$X$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Environment!$A$1:$X$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MASTER!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MASTER!$A$1:$X$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Mobility!$A$1:$X$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Water!$A$1:$X$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Weather!$A$1:$X$1</definedName>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3284" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3468" uniqueCount="806">
   <si>
     <t>Domain</t>
   </si>
@@ -2195,6 +2195,195 @@
   </si>
   <si>
     <t>16 routes — Refreshed every 2.5 min — Direct AI model input</t>
+  </si>
+  <si>
+    <t>Tram B</t>
+  </si>
+  <si>
+    <t>Network</t>
+  </si>
+  <si>
+    <t>TBM — GTFS Static (Routes + Stops + Timetable + Shapes)</t>
+  </si>
+  <si>
+    <t>tbm_gtfs_static</t>
+  </si>
+  <si>
+    <t>Full GTFS feed for TBM network — 207 routes, 5180 stops, 65340 trips, 66757 shape points. Filter route_short_name='B' for Tram B. Contains routes.txt, stops.txt, trips.txt, stop_times.txt, shapes.txt, calendar.txt, fare_products.txt.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83024</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/gtfsfeed/static/bordeaux?apiKey=opendata-bordeaux-metropole-flux-gtfs-rt</t>
+  </si>
+  <si>
+    <t>GTFS (ZIP)</t>
+  </si>
+  <si>
+    <t>LineString + Point</t>
+  </si>
+  <si>
+    <t>2026-05-29 to 2026-08-30</t>
+  </si>
+  <si>
+    <t>Licence Ouverte 1.0</t>
+  </si>
+  <si>
+    <t>TransitLine + TransitStop</t>
+  </si>
+  <si>
+    <t>TBM GTFS</t>
+  </si>
+  <si>
+    <t>Core static dataset — 20.99MB — filter route_short_name=B for Tram B only</t>
+  </si>
+  <si>
+    <t>Real-Time</t>
+  </si>
+  <si>
+    <t>TBM — GTFS-RT Vehicle Positions</t>
+  </si>
+  <si>
+    <t>tbm_gtfs_rt_vehicles</t>
+  </si>
+  <si>
+    <t>Real-time GPS positions of all TBM vehicles. Fields: vehicle_id, trip_id, route_id, latitude, longitude, bearing, speed, timestamp, currentStopSequence, currentStatus. Filter ineo-tram vehicles for Tram B.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83026</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/gtfsfeed/vehicles/bordeaux?apiKey=opendata-bordeaux-metropole-flux-gtfs-rt</t>
+  </si>
+  <si>
+    <t>GTFS-RT (Protobuf)</t>
+  </si>
+  <si>
+    <t>~30s</t>
+  </si>
+  <si>
+    <t>TBM GTFS-RT</t>
+  </si>
+  <si>
+    <t>KEY dataset for MiniTokyo3D animation — live tram position on track — 100% availability</t>
+  </si>
+  <si>
+    <t>TBM — GTFS-RT Trip Updates (Delays &amp; Cancellations)</t>
+  </si>
+  <si>
+    <t>tbm_gtfs_rt_tripupdates</t>
+  </si>
+  <si>
+    <t>Real-time trip updates for TBM network. Fields: trip_id, route_id, stop_id, arrival_delay, departure_delay, schedule_relationship. Used for ETA calculation and delay display per stop.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83025</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/gtfsfeed/realtime/bordeaux?apiKey=opendata-bordeaux-metropole-flux-gtfs-rt</t>
+  </si>
+  <si>
+    <t>trip_updates feed — delay in seconds per stop — 17 validation errors (minor)</t>
+  </si>
+  <si>
+    <t>TBM — GTFS-RT Service Alerts</t>
+  </si>
+  <si>
+    <t>tbm_gtfs_rt_alerts</t>
+  </si>
+  <si>
+    <t>Real-time service alerts for TBM network. Fields: alert_id, cause, effect, informed_entity (route/stop/trip), header_text, description_text, active_period. Covers relocated stops and unforeseen events.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83027</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/gtfsfeed/alerts/bordeaux?apiKey=opendata-bordeaux-metropole-flux-gtfs-rt</t>
+  </si>
+  <si>
+    <t>On event</t>
+  </si>
+  <si>
+    <t>TransitDiversion</t>
+  </si>
+  <si>
+    <t>service_alerts feed — no validation errors — display disruptions on DT dashboard</t>
+  </si>
+  <si>
+    <t>TBM — Route Geometry (sv_chem_l)</t>
+  </si>
+  <si>
+    <t>sv_chem_l_tramb</t>
+  </si>
+  <si>
+    <t>Geometric path of each TBM public transport line as GeoJSON LineString. Fields: ligne_id, ligne_nom, sens, distance, geometry. Filter ligne_nom='B' for Tram B route geometry on map.</t>
+  </si>
+  <si>
+    <t>TransitLine</t>
+  </si>
+  <si>
+    <t>Reference geometry for Tram B route — join with GTFS shapes.txt via ligne_id — essential for CesiumJS rendering</t>
+  </si>
+  <si>
+    <t>TBM — Physical Stops (sv_arret_p)</t>
+  </si>
+  <si>
+    <t>sv_arret_p_tramb</t>
+  </si>
+  <si>
+    <t>All physical stops (tram + bus) with location and attributes. Fields: arret_id, arret_nom, type_arret, pmr_acces, latitude, longitude, geometry. Filter type_arret='TRAM' for Tram B stops.</t>
+  </si>
+  <si>
+    <t>TransitStop</t>
+  </si>
+  <si>
+    <t>Stop reference for Tram B — join with GTFS stops.txt via stop_id — includes wheelchair accessibility</t>
+  </si>
+  <si>
+    <t>TBM — SIRI-Lite Stop Monitoring (Next Arrivals)</t>
+  </si>
+  <si>
+    <t>tbm_siri_stop_monitoring</t>
+  </si>
+  <si>
+    <t>Real-time arrival and departure times at a specific stop point. Fields: StopPointRef, LineRef, VehicleRef, AimedArrivalTime, ExpectedArrivalTime, AimedDepartureTime, ExpectedDepartureTime, Occupancy. Query per stop_id.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83031</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/siri/2.0/bordeaux/stop-monitoring.json?AccountKey=opendata-bordeaux-metropole-flux-gtfs-rt&amp;MonitoringRef=bordeaux:StopPoint:BP:STOP_ID:LOC</t>
+  </si>
+  <si>
+    <t>JSON (SIRI-Lite)</t>
+  </si>
+  <si>
+    <t>TBM SIRI-Lite</t>
+  </si>
+  <si>
+    <t>Next tram arrivals per station — replace STOP_ID in URL — key for station info panel in dashboard</t>
+  </si>
+  <si>
+    <t>Timetable</t>
+  </si>
+  <si>
+    <t>TBM — SIRI-Lite Estimated Timetable (Live Schedule)</t>
+  </si>
+  <si>
+    <t>tbm_siri_estimated_timetable</t>
+  </si>
+  <si>
+    <t>Calculated real-time timetable for a full line. Fields: LineRef, DirectionRef, DatedVehicleJourneyRef, StopPointRef, AimedArrivalTime, ExpectedArrivalTime, AimedDepartureTime, ExpectedDepartureTime. Query per line.</t>
+  </si>
+  <si>
+    <t>https://transport.data.gouv.fr/resources/83032</t>
+  </si>
+  <si>
+    <t>https://bdx.mecatran.com/utw/ws/siri/2.0/bordeaux/estimated-timetable.json?AccountKey=opendata-bordeaux-metropole-flux-gtfs-rt&amp;LineRef=bordeaux:Line:B:LOC&amp;DirectionRef=0</t>
+  </si>
+  <si>
+    <t>Full live timetable for Tram B — both directions (DirectionRef=0 and 1) — use for schedule panel</t>
   </si>
   <si>
     <t>domain</t>
@@ -2314,7 +2503,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2366,6 +2555,12 @@
         <fgColor rgb="FF9B59B6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -2379,7 +2574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2441,6 +2636,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2743,7 +2939,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X72"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:X80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3914,7 +4111,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>162</v>
       </c>
@@ -3986,7 +4183,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="18" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>162</v>
       </c>
@@ -4058,7 +4255,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>162</v>
       </c>
@@ -4130,7 +4327,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>162</v>
       </c>
@@ -4202,7 +4399,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>162</v>
       </c>
@@ -4274,7 +4471,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="22" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>162</v>
       </c>
@@ -4346,7 +4543,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="23" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>162</v>
       </c>
@@ -4418,7 +4615,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="24" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>162</v>
       </c>
@@ -4490,7 +4687,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>162</v>
       </c>
@@ -4562,7 +4759,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="26" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>162</v>
       </c>
@@ -4634,7 +4831,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="27" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>162</v>
       </c>
@@ -4706,7 +4903,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="28" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>162</v>
       </c>
@@ -4778,7 +4975,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="29" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>162</v>
       </c>
@@ -4850,7 +5047,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>162</v>
       </c>
@@ -4922,7 +5119,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="31" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>306</v>
       </c>
@@ -4992,7 +5189,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="32" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>306</v>
       </c>
@@ -5062,7 +5259,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="33" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>306</v>
       </c>
@@ -5134,7 +5331,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="34" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>306</v>
       </c>
@@ -5206,7 +5403,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="35" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>306</v>
       </c>
@@ -5278,7 +5475,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>306</v>
       </c>
@@ -5348,7 +5545,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>306</v>
       </c>
@@ -5418,7 +5615,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="38" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>306</v>
       </c>
@@ -5488,7 +5685,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="39" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>375</v>
       </c>
@@ -5558,7 +5755,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="40" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>375</v>
       </c>
@@ -5628,7 +5825,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="41" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
         <v>375</v>
       </c>
@@ -5698,7 +5895,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="42" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
         <v>375</v>
       </c>
@@ -5768,7 +5965,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="43" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
         <v>375</v>
       </c>
@@ -5838,7 +6035,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="44" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
         <v>375</v>
       </c>
@@ -5908,7 +6105,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="45" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>383</v>
       </c>
@@ -5980,7 +6177,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="46" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>383</v>
       </c>
@@ -6052,7 +6249,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="47" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>383</v>
       </c>
@@ -6122,7 +6319,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="48" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>383</v>
       </c>
@@ -6192,7 +6389,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="49" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="6" t="s">
         <v>383</v>
       </c>
@@ -6262,7 +6459,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="50" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="6" t="s">
         <v>383</v>
       </c>
@@ -6332,7 +6529,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="51" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="6" t="s">
         <v>383</v>
       </c>
@@ -6402,7 +6599,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="52" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>375</v>
       </c>
@@ -6472,7 +6669,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="53" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
         <v>507</v>
       </c>
@@ -6542,7 +6739,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="54" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
         <v>522</v>
       </c>
@@ -6612,7 +6809,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="55" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
         <v>522</v>
       </c>
@@ -6682,7 +6879,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="56" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="13" t="s">
         <v>522</v>
       </c>
@@ -6754,7 +6951,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="57" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="13" t="s">
         <v>522</v>
       </c>
@@ -6824,7 +7021,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="58" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="13" t="s">
         <v>522</v>
       </c>
@@ -6896,7 +7093,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="59" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="13" t="s">
         <v>522</v>
       </c>
@@ -6968,7 +7165,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="60" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="13" t="s">
         <v>522</v>
       </c>
@@ -7038,7 +7235,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="61" spans="1:24" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:24" ht="24" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="13" t="s">
         <v>522</v>
       </c>
@@ -7110,7 +7307,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="62" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="13" t="s">
         <v>522</v>
       </c>
@@ -7180,7 +7377,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="63" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="14" t="s">
         <v>622</v>
       </c>
@@ -7250,7 +7447,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="64" spans="1:24" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:24" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="14" t="s">
         <v>622</v>
       </c>
@@ -7320,7 +7517,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="65" spans="1:24" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:24" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="14" t="s">
         <v>622</v>
       </c>
@@ -7390,7 +7587,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="66" spans="1:24" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:24" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="14" t="s">
         <v>622</v>
       </c>
@@ -7460,7 +7657,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="67" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>664</v>
       </c>
@@ -7532,7 +7729,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="68" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>664</v>
       </c>
@@ -7604,7 +7801,7 @@
         <v>683</v>
       </c>
     </row>
-    <row r="69" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>684</v>
       </c>
@@ -7676,7 +7873,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="70" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>684</v>
       </c>
@@ -7748,7 +7945,7 @@
         <v>703</v>
       </c>
     </row>
-    <row r="71" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>684</v>
       </c>
@@ -7820,7 +8017,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="72" spans="1:24" ht="36" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:24" ht="36" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>684</v>
       </c>
@@ -7892,8 +8089,582 @@
         <v>718</v>
       </c>
     </row>
+    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A73" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B73" t="s">
+        <v>720</v>
+      </c>
+      <c r="C73" t="s">
+        <v>721</v>
+      </c>
+      <c r="D73" t="s">
+        <v>722</v>
+      </c>
+      <c r="E73" t="s">
+        <v>72</v>
+      </c>
+      <c r="F73" t="s">
+        <v>723</v>
+      </c>
+      <c r="G73" t="s">
+        <v>724</v>
+      </c>
+      <c r="I73" t="s">
+        <v>725</v>
+      </c>
+      <c r="J73" t="s">
+        <v>726</v>
+      </c>
+      <c r="K73" t="s">
+        <v>727</v>
+      </c>
+      <c r="L73" t="s">
+        <v>132</v>
+      </c>
+      <c r="M73" t="s">
+        <v>132</v>
+      </c>
+      <c r="N73" t="s">
+        <v>728</v>
+      </c>
+      <c r="O73" t="s">
+        <v>28</v>
+      </c>
+      <c r="P73" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>38</v>
+      </c>
+      <c r="R73" t="s">
+        <v>39</v>
+      </c>
+      <c r="S73" t="s">
+        <v>39</v>
+      </c>
+      <c r="T73" t="s">
+        <v>40</v>
+      </c>
+      <c r="U73" t="s">
+        <v>730</v>
+      </c>
+      <c r="V73" t="s">
+        <v>731</v>
+      </c>
+      <c r="W73" t="s">
+        <v>72</v>
+      </c>
+      <c r="X73" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A74" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B74" t="s">
+        <v>733</v>
+      </c>
+      <c r="C74" t="s">
+        <v>734</v>
+      </c>
+      <c r="D74" t="s">
+        <v>735</v>
+      </c>
+      <c r="E74" t="s">
+        <v>72</v>
+      </c>
+      <c r="F74" t="s">
+        <v>736</v>
+      </c>
+      <c r="G74" t="s">
+        <v>737</v>
+      </c>
+      <c r="H74" t="s">
+        <v>738</v>
+      </c>
+      <c r="J74" t="s">
+        <v>739</v>
+      </c>
+      <c r="K74" t="s">
+        <v>49</v>
+      </c>
+      <c r="L74" t="s">
+        <v>34</v>
+      </c>
+      <c r="M74" t="s">
+        <v>740</v>
+      </c>
+      <c r="N74" t="s">
+        <v>36</v>
+      </c>
+      <c r="O74" t="s">
+        <v>28</v>
+      </c>
+      <c r="P74" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>38</v>
+      </c>
+      <c r="R74" t="s">
+        <v>39</v>
+      </c>
+      <c r="S74" t="s">
+        <v>39</v>
+      </c>
+      <c r="T74" t="s">
+        <v>40</v>
+      </c>
+      <c r="U74" t="s">
+        <v>87</v>
+      </c>
+      <c r="V74" t="s">
+        <v>741</v>
+      </c>
+      <c r="W74" t="s">
+        <v>72</v>
+      </c>
+      <c r="X74" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A75" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B75" t="s">
+        <v>733</v>
+      </c>
+      <c r="C75" t="s">
+        <v>743</v>
+      </c>
+      <c r="D75" t="s">
+        <v>744</v>
+      </c>
+      <c r="E75" t="s">
+        <v>72</v>
+      </c>
+      <c r="F75" t="s">
+        <v>745</v>
+      </c>
+      <c r="G75" t="s">
+        <v>746</v>
+      </c>
+      <c r="H75" t="s">
+        <v>747</v>
+      </c>
+      <c r="J75" t="s">
+        <v>739</v>
+      </c>
+      <c r="K75" t="s">
+        <v>154</v>
+      </c>
+      <c r="L75" t="s">
+        <v>34</v>
+      </c>
+      <c r="M75" t="s">
+        <v>740</v>
+      </c>
+      <c r="N75" t="s">
+        <v>36</v>
+      </c>
+      <c r="O75" t="s">
+        <v>28</v>
+      </c>
+      <c r="P75" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>38</v>
+      </c>
+      <c r="R75" t="s">
+        <v>39</v>
+      </c>
+      <c r="S75" t="s">
+        <v>39</v>
+      </c>
+      <c r="T75" t="s">
+        <v>40</v>
+      </c>
+      <c r="U75" t="s">
+        <v>717</v>
+      </c>
+      <c r="V75" t="s">
+        <v>741</v>
+      </c>
+      <c r="W75" t="s">
+        <v>72</v>
+      </c>
+      <c r="X75" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A76" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B76" t="s">
+        <v>733</v>
+      </c>
+      <c r="C76" t="s">
+        <v>749</v>
+      </c>
+      <c r="D76" t="s">
+        <v>750</v>
+      </c>
+      <c r="E76" t="s">
+        <v>72</v>
+      </c>
+      <c r="F76" t="s">
+        <v>751</v>
+      </c>
+      <c r="G76" t="s">
+        <v>752</v>
+      </c>
+      <c r="H76" t="s">
+        <v>753</v>
+      </c>
+      <c r="J76" t="s">
+        <v>739</v>
+      </c>
+      <c r="K76" t="s">
+        <v>154</v>
+      </c>
+      <c r="L76" t="s">
+        <v>34</v>
+      </c>
+      <c r="M76" t="s">
+        <v>754</v>
+      </c>
+      <c r="N76" t="s">
+        <v>36</v>
+      </c>
+      <c r="O76" t="s">
+        <v>28</v>
+      </c>
+      <c r="P76" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>38</v>
+      </c>
+      <c r="R76" t="s">
+        <v>39</v>
+      </c>
+      <c r="S76" t="s">
+        <v>108</v>
+      </c>
+      <c r="T76" t="s">
+        <v>51</v>
+      </c>
+      <c r="U76" t="s">
+        <v>755</v>
+      </c>
+      <c r="V76" t="s">
+        <v>741</v>
+      </c>
+      <c r="W76" t="s">
+        <v>72</v>
+      </c>
+      <c r="X76" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A77" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B77" t="s">
+        <v>720</v>
+      </c>
+      <c r="C77" t="s">
+        <v>757</v>
+      </c>
+      <c r="D77" t="s">
+        <v>758</v>
+      </c>
+      <c r="E77" t="s">
+        <v>28</v>
+      </c>
+      <c r="F77" t="s">
+        <v>759</v>
+      </c>
+      <c r="G77" t="s">
+        <v>66</v>
+      </c>
+      <c r="H77" t="s">
+        <v>67</v>
+      </c>
+      <c r="J77" t="s">
+        <v>32</v>
+      </c>
+      <c r="K77" t="s">
+        <v>33</v>
+      </c>
+      <c r="L77" t="s">
+        <v>68</v>
+      </c>
+      <c r="M77" t="s">
+        <v>69</v>
+      </c>
+      <c r="N77" t="s">
+        <v>36</v>
+      </c>
+      <c r="O77" t="s">
+        <v>28</v>
+      </c>
+      <c r="P77" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>38</v>
+      </c>
+      <c r="R77" t="s">
+        <v>39</v>
+      </c>
+      <c r="S77" t="s">
+        <v>39</v>
+      </c>
+      <c r="T77" t="s">
+        <v>40</v>
+      </c>
+      <c r="U77" t="s">
+        <v>760</v>
+      </c>
+      <c r="V77" t="s">
+        <v>71</v>
+      </c>
+      <c r="W77" t="s">
+        <v>72</v>
+      </c>
+      <c r="X77" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="78" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A78" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B78" t="s">
+        <v>720</v>
+      </c>
+      <c r="C78" t="s">
+        <v>762</v>
+      </c>
+      <c r="D78" t="s">
+        <v>763</v>
+      </c>
+      <c r="E78" t="s">
+        <v>28</v>
+      </c>
+      <c r="F78" t="s">
+        <v>764</v>
+      </c>
+      <c r="G78" t="s">
+        <v>99</v>
+      </c>
+      <c r="H78" t="s">
+        <v>100</v>
+      </c>
+      <c r="J78" t="s">
+        <v>32</v>
+      </c>
+      <c r="K78" t="s">
+        <v>49</v>
+      </c>
+      <c r="L78" t="s">
+        <v>68</v>
+      </c>
+      <c r="M78" t="s">
+        <v>69</v>
+      </c>
+      <c r="N78" t="s">
+        <v>36</v>
+      </c>
+      <c r="O78" t="s">
+        <v>28</v>
+      </c>
+      <c r="P78" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>38</v>
+      </c>
+      <c r="R78" t="s">
+        <v>39</v>
+      </c>
+      <c r="S78" t="s">
+        <v>39</v>
+      </c>
+      <c r="T78" t="s">
+        <v>40</v>
+      </c>
+      <c r="U78" t="s">
+        <v>765</v>
+      </c>
+      <c r="V78" t="s">
+        <v>71</v>
+      </c>
+      <c r="W78" t="s">
+        <v>72</v>
+      </c>
+      <c r="X78" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="79" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A79" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B79" t="s">
+        <v>733</v>
+      </c>
+      <c r="C79" t="s">
+        <v>767</v>
+      </c>
+      <c r="D79" t="s">
+        <v>768</v>
+      </c>
+      <c r="E79" t="s">
+        <v>72</v>
+      </c>
+      <c r="F79" t="s">
+        <v>769</v>
+      </c>
+      <c r="G79" t="s">
+        <v>770</v>
+      </c>
+      <c r="H79" t="s">
+        <v>771</v>
+      </c>
+      <c r="J79" t="s">
+        <v>772</v>
+      </c>
+      <c r="K79" t="s">
+        <v>154</v>
+      </c>
+      <c r="L79" t="s">
+        <v>34</v>
+      </c>
+      <c r="M79" t="s">
+        <v>740</v>
+      </c>
+      <c r="N79" t="s">
+        <v>36</v>
+      </c>
+      <c r="O79" t="s">
+        <v>28</v>
+      </c>
+      <c r="P79" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>38</v>
+      </c>
+      <c r="R79" t="s">
+        <v>39</v>
+      </c>
+      <c r="S79" t="s">
+        <v>39</v>
+      </c>
+      <c r="T79" t="s">
+        <v>40</v>
+      </c>
+      <c r="U79" t="s">
+        <v>87</v>
+      </c>
+      <c r="V79" t="s">
+        <v>773</v>
+      </c>
+      <c r="W79" t="s">
+        <v>72</v>
+      </c>
+      <c r="X79" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="80" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A80" s="21" t="s">
+        <v>719</v>
+      </c>
+      <c r="B80" t="s">
+        <v>775</v>
+      </c>
+      <c r="C80" t="s">
+        <v>776</v>
+      </c>
+      <c r="D80" t="s">
+        <v>777</v>
+      </c>
+      <c r="E80" t="s">
+        <v>72</v>
+      </c>
+      <c r="F80" t="s">
+        <v>778</v>
+      </c>
+      <c r="G80" t="s">
+        <v>779</v>
+      </c>
+      <c r="H80" t="s">
+        <v>780</v>
+      </c>
+      <c r="J80" t="s">
+        <v>772</v>
+      </c>
+      <c r="K80" t="s">
+        <v>154</v>
+      </c>
+      <c r="L80" t="s">
+        <v>34</v>
+      </c>
+      <c r="M80" t="s">
+        <v>740</v>
+      </c>
+      <c r="N80" t="s">
+        <v>36</v>
+      </c>
+      <c r="O80" t="s">
+        <v>28</v>
+      </c>
+      <c r="P80" t="s">
+        <v>729</v>
+      </c>
+      <c r="Q80" t="s">
+        <v>38</v>
+      </c>
+      <c r="R80" t="s">
+        <v>39</v>
+      </c>
+      <c r="S80" t="s">
+        <v>39</v>
+      </c>
+      <c r="T80" t="s">
+        <v>51</v>
+      </c>
+      <c r="U80" t="s">
+        <v>717</v>
+      </c>
+      <c r="V80" t="s">
+        <v>773</v>
+      </c>
+      <c r="W80" t="s">
+        <v>72</v>
+      </c>
+      <c r="X80" t="s">
+        <v>781</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:X1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:X72" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Mobility"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12088,76 +12859,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="15" t="s">
-        <v>719</v>
+        <v>782</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>720</v>
+        <v>783</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>721</v>
+        <v>784</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>722</v>
+        <v>785</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>723</v>
+        <v>786</v>
       </c>
       <c r="F1" s="15" t="s">
-        <v>724</v>
+        <v>787</v>
       </c>
       <c r="G1" s="15" t="s">
-        <v>725</v>
+        <v>788</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>726</v>
+        <v>789</v>
       </c>
       <c r="I1" s="15" t="s">
-        <v>727</v>
+        <v>790</v>
       </c>
       <c r="J1" s="15" t="s">
-        <v>728</v>
+        <v>791</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>729</v>
+        <v>792</v>
       </c>
       <c r="L1" s="15" t="s">
-        <v>730</v>
+        <v>793</v>
       </c>
       <c r="M1" s="15" t="s">
-        <v>731</v>
+        <v>794</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>732</v>
+        <v>795</v>
       </c>
       <c r="O1" s="15" t="s">
-        <v>733</v>
+        <v>796</v>
       </c>
       <c r="P1" s="15" t="s">
-        <v>734</v>
+        <v>797</v>
       </c>
       <c r="Q1" s="15" t="s">
-        <v>735</v>
+        <v>798</v>
       </c>
       <c r="R1" s="15" t="s">
-        <v>736</v>
+        <v>799</v>
       </c>
       <c r="S1" s="15" t="s">
-        <v>737</v>
+        <v>800</v>
       </c>
       <c r="T1" s="15" t="s">
-        <v>738</v>
+        <v>801</v>
       </c>
       <c r="U1" s="15" t="s">
-        <v>739</v>
+        <v>802</v>
       </c>
       <c r="V1" s="15" t="s">
-        <v>740</v>
+        <v>803</v>
       </c>
       <c r="W1" s="15" t="s">
-        <v>741</v>
+        <v>804</v>
       </c>
       <c r="X1" s="15" t="s">
-        <v>742</v>
+        <v>805</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -12247,76 +13018,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
-        <v>719</v>
+        <v>782</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>720</v>
+        <v>783</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>721</v>
+        <v>784</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>722</v>
+        <v>785</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>723</v>
+        <v>786</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>724</v>
+        <v>787</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>725</v>
+        <v>788</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>726</v>
+        <v>789</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>727</v>
+        <v>790</v>
       </c>
       <c r="J1" s="16" t="s">
-        <v>728</v>
+        <v>791</v>
       </c>
       <c r="K1" s="16" t="s">
-        <v>729</v>
+        <v>792</v>
       </c>
       <c r="L1" s="16" t="s">
-        <v>730</v>
+        <v>793</v>
       </c>
       <c r="M1" s="16" t="s">
-        <v>731</v>
+        <v>794</v>
       </c>
       <c r="N1" s="16" t="s">
-        <v>732</v>
+        <v>795</v>
       </c>
       <c r="O1" s="16" t="s">
-        <v>733</v>
+        <v>796</v>
       </c>
       <c r="P1" s="16" t="s">
-        <v>734</v>
+        <v>797</v>
       </c>
       <c r="Q1" s="16" t="s">
-        <v>735</v>
+        <v>798</v>
       </c>
       <c r="R1" s="16" t="s">
-        <v>736</v>
+        <v>799</v>
       </c>
       <c r="S1" s="16" t="s">
-        <v>737</v>
+        <v>800</v>
       </c>
       <c r="T1" s="16" t="s">
-        <v>738</v>
+        <v>801</v>
       </c>
       <c r="U1" s="16" t="s">
-        <v>739</v>
+        <v>802</v>
       </c>
       <c r="V1" s="16" t="s">
-        <v>740</v>
+        <v>803</v>
       </c>
       <c r="W1" s="16" t="s">
-        <v>741</v>
+        <v>804</v>
       </c>
       <c r="X1" s="16" t="s">
-        <v>742</v>
+        <v>805</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="168" customHeight="1" x14ac:dyDescent="0.3">
@@ -12975,76 +13746,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="17" t="s">
-        <v>719</v>
+        <v>782</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>720</v>
+        <v>783</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>721</v>
+        <v>784</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>722</v>
+        <v>785</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>723</v>
+        <v>786</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>724</v>
+        <v>787</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>725</v>
+        <v>788</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>726</v>
+        <v>789</v>
       </c>
       <c r="I1" s="17" t="s">
-        <v>727</v>
+        <v>790</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>728</v>
+        <v>791</v>
       </c>
       <c r="K1" s="17" t="s">
-        <v>729</v>
+        <v>792</v>
       </c>
       <c r="L1" s="17" t="s">
-        <v>730</v>
+        <v>793</v>
       </c>
       <c r="M1" s="17" t="s">
-        <v>731</v>
+        <v>794</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>732</v>
+        <v>795</v>
       </c>
       <c r="O1" s="17" t="s">
-        <v>733</v>
+        <v>796</v>
       </c>
       <c r="P1" s="17" t="s">
-        <v>734</v>
+        <v>797</v>
       </c>
       <c r="Q1" s="17" t="s">
-        <v>735</v>
+        <v>798</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>736</v>
+        <v>799</v>
       </c>
       <c r="S1" s="17" t="s">
-        <v>737</v>
+        <v>800</v>
       </c>
       <c r="T1" s="17" t="s">
-        <v>738</v>
+        <v>801</v>
       </c>
       <c r="U1" s="17" t="s">
-        <v>739</v>
+        <v>802</v>
       </c>
       <c r="V1" s="17" t="s">
-        <v>740</v>
+        <v>803</v>
       </c>
       <c r="W1" s="17" t="s">
-        <v>741</v>
+        <v>804</v>
       </c>
       <c r="X1" s="17" t="s">
-        <v>742</v>
+        <v>805</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="70.2" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>